<commit_message>
3 - Começo do Tratamento de Dados
Começo do tratamento de dados, onde inicio pela coluna data.
</commit_message>
<xml_diff>
--- a/data/dados_tratados.xlsx
+++ b/data/dados_tratados.xlsx
@@ -8,24 +8,38 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\analise-vendas-excel\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB6E3192-A080-40BD-B095-EC3E0D9920E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0E82B7F-B388-4B88-AEDA-F6ECEA6C729D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dados Tratados" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dados Tratados'!$A$1:$G$121</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="174">
   <si>
     <t>Data</t>
   </si>
@@ -48,9 +62,6 @@
     <t>Receita</t>
   </si>
   <si>
-    <t>03-08-2023</t>
-  </si>
-  <si>
     <t>Monitor</t>
   </si>
   <si>
@@ -63,9 +74,6 @@
     <t>40810.25</t>
   </si>
   <si>
-    <t>2023-04-25</t>
-  </si>
-  <si>
     <t>Notebook</t>
   </si>
   <si>
@@ -75,69 +83,39 @@
     <t>Carlos</t>
   </si>
   <si>
-    <t>2023-02-09 00:00:00</t>
-  </si>
-  <si>
     <t>sul</t>
   </si>
   <si>
     <t>Daniela</t>
   </si>
   <si>
-    <t>2023-07-04 00:00:00</t>
-  </si>
-  <si>
     <t>Teclado</t>
   </si>
   <si>
     <t xml:space="preserve"> Sudeste </t>
   </si>
   <si>
-    <t>01-17-2023</t>
-  </si>
-  <si>
     <t>Headset</t>
   </si>
   <si>
     <t>Bruno</t>
   </si>
   <si>
-    <t>R$ 760.94</t>
-  </si>
-  <si>
-    <t>2023-12-28</t>
-  </si>
-  <si>
     <t>CENTRO-OESTE</t>
   </si>
   <si>
-    <t>2023-10-26 00:00:00</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Sul </t>
   </si>
   <si>
     <t>11 unidades</t>
   </si>
   <si>
-    <t>2465,45</t>
-  </si>
-  <si>
     <t>46843.55</t>
   </si>
   <si>
-    <t>2023-01-07</t>
-  </si>
-  <si>
     <t>1 unidades</t>
   </si>
   <si>
-    <t>758,5</t>
-  </si>
-  <si>
-    <t>12-03-2023</t>
-  </si>
-  <si>
     <t>centro-oeste</t>
   </si>
   <si>
@@ -147,48 +125,27 @@
     <t>10834.45</t>
   </si>
   <si>
-    <t>2023-12-16 00:00:00</t>
-  </si>
-  <si>
     <t>Ana</t>
   </si>
   <si>
     <t>3 unidades</t>
   </si>
   <si>
-    <t>2649,97</t>
-  </si>
-  <si>
-    <t>2023-01-12</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Centro-Oeste </t>
   </si>
   <si>
     <t>6 unidades</t>
   </si>
   <si>
-    <t>1855,07</t>
-  </si>
-  <si>
-    <t>14/02/2023</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Nordeste </t>
   </si>
   <si>
     <t>2 unidades</t>
   </si>
   <si>
-    <t>4836,45</t>
-  </si>
-  <si>
     <t>91892.55</t>
   </si>
   <si>
-    <t>2023-07-24 00:00:00</t>
-  </si>
-  <si>
     <t>5 unidades</t>
   </si>
   <si>
@@ -198,12 +155,6 @@
     <t>51987.0</t>
   </si>
   <si>
-    <t>2023-01-11</t>
-  </si>
-  <si>
-    <t>4133,85</t>
-  </si>
-  <si>
     <t>37204.65</t>
   </si>
   <si>
@@ -213,30 +164,18 @@
     <t>R$ 2905.81</t>
   </si>
   <si>
-    <t>2023-04-21 00:00:00</t>
-  </si>
-  <si>
-    <t>09-19-2023</t>
-  </si>
-  <si>
     <t>865,64</t>
   </si>
   <si>
     <t>5193.84</t>
   </si>
   <si>
-    <t>2023-09-08 00:00:00</t>
-  </si>
-  <si>
     <t>19 unidades</t>
   </si>
   <si>
     <t>R$ 2275.71</t>
   </si>
   <si>
-    <t>2023-04-20</t>
-  </si>
-  <si>
     <t>sudeste</t>
   </si>
   <si>
@@ -246,18 +185,12 @@
     <t>192,09</t>
   </si>
   <si>
-    <t>07/07/2023</t>
-  </si>
-  <si>
     <t>8 unidades</t>
   </si>
   <si>
     <t>1582,95</t>
   </si>
   <si>
-    <t>2023-02-22 00:00:00</t>
-  </si>
-  <si>
     <t>NORDESTE</t>
   </si>
   <si>
@@ -270,9 +203,6 @@
     <t>14855.8</t>
   </si>
   <si>
-    <t>20/12/2023</t>
-  </si>
-  <si>
     <t>Mouse</t>
   </si>
   <si>
@@ -285,27 +215,18 @@
     <t>97991.8</t>
   </si>
   <si>
-    <t>19/05/2023</t>
-  </si>
-  <si>
     <t>SUL</t>
   </si>
   <si>
     <t>R$ 717.83</t>
   </si>
   <si>
-    <t>14/06/2023</t>
-  </si>
-  <si>
     <t>14 unidades</t>
   </si>
   <si>
     <t>R$ 2077.83</t>
   </si>
   <si>
-    <t>14/07/2023</t>
-  </si>
-  <si>
     <t>17 unidades</t>
   </si>
   <si>
@@ -315,9 +236,6 @@
     <t>6717.87</t>
   </si>
   <si>
-    <t>2023-10-06 00:00:00</t>
-  </si>
-  <si>
     <t>nordeste</t>
   </si>
   <si>
@@ -327,12 +245,6 @@
     <t>1087,75</t>
   </si>
   <si>
-    <t>10/02/2023</t>
-  </si>
-  <si>
-    <t>26/09/2023</t>
-  </si>
-  <si>
     <t>13 unidades</t>
   </si>
   <si>
@@ -342,54 +254,30 @@
     <t>3123.27</t>
   </si>
   <si>
-    <t>06-24-2023</t>
-  </si>
-  <si>
     <t>R$ 4913.28</t>
   </si>
   <si>
-    <t>03-27-2023</t>
-  </si>
-  <si>
     <t>R$ 1390.01</t>
   </si>
   <si>
-    <t>26/05/2023</t>
-  </si>
-  <si>
     <t>R$ 3523.1</t>
   </si>
   <si>
     <t>10569.3</t>
   </si>
   <si>
-    <t>2023-06-29 00:00:00</t>
-  </si>
-  <si>
     <t>83244.24</t>
   </si>
   <si>
-    <t>16/02/2023</t>
-  </si>
-  <si>
     <t>R$ 3596.45</t>
   </si>
   <si>
     <t>R$ 1401.69</t>
   </si>
   <si>
-    <t>05-22-2023</t>
-  </si>
-  <si>
     <t>R$ 2415.07</t>
   </si>
   <si>
-    <t>2023-06-14 00:00:00</t>
-  </si>
-  <si>
-    <t>2023-01-28 00:00:00</t>
-  </si>
-  <si>
     <t>SUDESTE</t>
   </si>
   <si>
@@ -399,342 +287,180 @@
     <t>17154.55</t>
   </si>
   <si>
-    <t>2023-04-04 00:00:00</t>
-  </si>
-  <si>
     <t>6772.8</t>
   </si>
   <si>
-    <t>19/10/2023</t>
-  </si>
-  <si>
     <t>R$ 3629.92</t>
   </si>
   <si>
-    <t>2023-10-27 00:00:00</t>
-  </si>
-  <si>
     <t>636,05</t>
   </si>
   <si>
     <t>6360.5</t>
   </si>
   <si>
-    <t>14/08/2023</t>
-  </si>
-  <si>
-    <t>2023-05-23 00:00:00</t>
-  </si>
-  <si>
     <t>3710,43</t>
   </si>
   <si>
-    <t>04-11-2023</t>
-  </si>
-  <si>
     <t>1012,69</t>
   </si>
   <si>
-    <t>2023-03-14</t>
-  </si>
-  <si>
-    <t>25/07/2023</t>
-  </si>
-  <si>
     <t>384,76</t>
   </si>
   <si>
     <t>4617.12</t>
   </si>
   <si>
-    <t>2023-10-20 00:00:00</t>
-  </si>
-  <si>
     <t>R$ 550.23</t>
   </si>
   <si>
-    <t>2023-12-13</t>
-  </si>
-  <si>
     <t>2683,74</t>
   </si>
   <si>
-    <t>08-02-2023</t>
-  </si>
-  <si>
     <t>R$ 4961.6</t>
   </si>
   <si>
-    <t>2023-08-10 00:00:00</t>
-  </si>
-  <si>
     <t>R$ 3624.34</t>
   </si>
   <si>
-    <t>18/02/2023</t>
-  </si>
-  <si>
-    <t>02-20-2023</t>
-  </si>
-  <si>
-    <t>12-20-2023</t>
-  </si>
-  <si>
     <t>R$ 482.06</t>
   </si>
   <si>
-    <t>12-14-2023</t>
-  </si>
-  <si>
     <t>R$ 1424.69</t>
   </si>
   <si>
-    <t>13/09/2023</t>
-  </si>
-  <si>
     <t>3822,16</t>
   </si>
   <si>
-    <t>09-25-2023</t>
-  </si>
-  <si>
     <t>90,35</t>
   </si>
   <si>
-    <t>2023-11-12</t>
-  </si>
-  <si>
     <t>1966,9</t>
   </si>
   <si>
-    <t>2023-08-08</t>
-  </si>
-  <si>
     <t>1211.28</t>
   </si>
   <si>
-    <t>2023-04-12</t>
-  </si>
-  <si>
     <t>9919.56</t>
   </si>
   <si>
-    <t>2023-08-23 00:00:00</t>
-  </si>
-  <si>
     <t>R$ 4615.97</t>
   </si>
   <si>
     <t>9231.94</t>
   </si>
   <si>
-    <t>2023-02-08</t>
-  </si>
-  <si>
-    <t>08-31-2023</t>
-  </si>
-  <si>
     <t>3407,04</t>
   </si>
   <si>
     <t>10221.12</t>
   </si>
   <si>
-    <t>2023-10-19</t>
-  </si>
-  <si>
-    <t>2023-05-06</t>
-  </si>
-  <si>
-    <t>2023-08-17</t>
-  </si>
-  <si>
     <t>R$ 807.99</t>
   </si>
   <si>
-    <t>05/01/2023</t>
-  </si>
-  <si>
     <t>2331,2</t>
   </si>
   <si>
-    <t>2023-12-31</t>
-  </si>
-  <si>
     <t>2293,25</t>
   </si>
   <si>
-    <t>02-02-2023</t>
-  </si>
-  <si>
     <t>15 unidades</t>
   </si>
   <si>
     <t>R$ 3908.7</t>
   </si>
   <si>
-    <t>2023-07-21 00:00:00</t>
-  </si>
-  <si>
     <t>R$ 2016.18</t>
   </si>
   <si>
     <t>10080.9</t>
   </si>
   <si>
-    <t>2023-09-18</t>
-  </si>
-  <si>
     <t>1077,94</t>
   </si>
   <si>
-    <t>2023-09-27 00:00:00</t>
-  </si>
-  <si>
     <t>2196,89</t>
   </si>
   <si>
-    <t>2023-05-16 00:00:00</t>
-  </si>
-  <si>
     <t>R$ 3923.26</t>
   </si>
   <si>
-    <t>12-26-2023</t>
-  </si>
-  <si>
     <t>R$ 2643.65</t>
   </si>
   <si>
     <t>37011.1</t>
   </si>
   <si>
-    <t>2023-08-31</t>
-  </si>
-  <si>
     <t>R$ 3587.68</t>
   </si>
   <si>
     <t>21526.08</t>
   </si>
   <si>
-    <t>01-18-2023</t>
-  </si>
-  <si>
     <t>3728,53</t>
   </si>
   <si>
-    <t>10-12-2023</t>
-  </si>
-  <si>
     <t>R$ 313.21</t>
   </si>
   <si>
-    <t>24/05/2023</t>
-  </si>
-  <si>
     <t>R$ 295.97</t>
   </si>
   <si>
-    <t>12/06/2023</t>
-  </si>
-  <si>
     <t>R$ 1882.81</t>
   </si>
   <si>
     <t>24476.53</t>
   </si>
   <si>
-    <t>07/10/2023</t>
-  </si>
-  <si>
     <t>27818.31</t>
   </si>
   <si>
-    <t>2023-03-31</t>
-  </si>
-  <si>
     <t>12 unidades</t>
   </si>
   <si>
     <t>4698,22</t>
   </si>
   <si>
-    <t>06-09-2023</t>
-  </si>
-  <si>
     <t>R$ 4513.9</t>
   </si>
   <si>
     <t>85764.1</t>
   </si>
   <si>
-    <t>11-21-2023</t>
-  </si>
-  <si>
     <t>1524,53</t>
   </si>
   <si>
-    <t>05-12-2023</t>
-  </si>
-  <si>
     <t>R$ 3318.1</t>
   </si>
   <si>
-    <t>21/01/2023</t>
-  </si>
-  <si>
     <t>2418,33</t>
   </si>
   <si>
-    <t>2023-02-23 00:00:00</t>
-  </si>
-  <si>
-    <t>2023-04-24</t>
-  </si>
-  <si>
     <t>645,74</t>
   </si>
   <si>
     <t>10331.84</t>
   </si>
   <si>
-    <t>2023-09-13 00:00:00</t>
-  </si>
-  <si>
     <t>111,36</t>
   </si>
   <si>
-    <t>2023-02-24 00:00:00</t>
-  </si>
-  <si>
     <t>R$ 130.11</t>
   </si>
   <si>
-    <t>2023-10-14 00:00:00</t>
-  </si>
-  <si>
     <t>3838,04</t>
   </si>
   <si>
     <t>3838.04</t>
   </si>
   <si>
-    <t>2023-07-26</t>
-  </si>
-  <si>
     <t>1595,86</t>
   </si>
   <si>
     <t>1595.86</t>
   </si>
   <si>
-    <t>2023-07-26 00:00:00</t>
-  </si>
-  <si>
-    <t>2023-04-13 00:00:00</t>
-  </si>
-  <si>
     <t>2787,97</t>
   </si>
   <si>
@@ -747,156 +473,81 @@
     <t>26996.94</t>
   </si>
   <si>
-    <t>11-18-2023</t>
-  </si>
-  <si>
     <t>R$ 1651.42</t>
   </si>
   <si>
-    <t>2023-06-16</t>
-  </si>
-  <si>
     <t>R$ 2505.55</t>
   </si>
   <si>
-    <t>06/04/2023</t>
-  </si>
-  <si>
     <t>4433,57</t>
   </si>
   <si>
-    <t>02/02/2023</t>
-  </si>
-  <si>
-    <t>20/06/2023</t>
-  </si>
-  <si>
     <t>2078,11</t>
   </si>
   <si>
-    <t>2023-03-27</t>
-  </si>
-  <si>
     <t>4 unidades</t>
   </si>
   <si>
     <t>9328.53</t>
   </si>
   <si>
-    <t>2023-11-23 00:00:00</t>
-  </si>
-  <si>
     <t>12563.04</t>
   </si>
   <si>
-    <t>2023-06-09 00:00:00</t>
-  </si>
-  <si>
     <t>R$ 1168.19</t>
   </si>
   <si>
     <t>8177.33</t>
   </si>
   <si>
-    <t>2023-08-12</t>
-  </si>
-  <si>
     <t>R$ 2136.39</t>
   </si>
   <si>
-    <t>08/07/2023</t>
-  </si>
-  <si>
     <t>4775,7</t>
   </si>
   <si>
     <t>33429.9</t>
   </si>
   <si>
-    <t>20/11/2023</t>
-  </si>
-  <si>
     <t>3978,43</t>
   </si>
   <si>
     <t>47741.16</t>
   </si>
   <si>
-    <t>09-04-2023</t>
-  </si>
-  <si>
-    <t>11/04/2023</t>
-  </si>
-  <si>
     <t>179,65</t>
   </si>
   <si>
     <t>2155.8</t>
   </si>
   <si>
-    <t>2023-06-08</t>
-  </si>
-  <si>
     <t>R$ 573.21</t>
   </si>
   <si>
-    <t>10-29-2023</t>
-  </si>
-  <si>
-    <t>2023-12-24 00:00:00</t>
-  </si>
-  <si>
-    <t>2023-11-20 00:00:00</t>
-  </si>
-  <si>
-    <t>02-26-2023</t>
-  </si>
-  <si>
-    <t>1348,91</t>
-  </si>
-  <si>
-    <t>12/03/2023</t>
-  </si>
-  <si>
     <t>51491.52</t>
   </si>
   <si>
-    <t>03/05/2023</t>
-  </si>
-  <si>
     <t>6073.8</t>
   </si>
   <si>
-    <t>10-08-2023</t>
-  </si>
-  <si>
     <t>R$ 1650.85</t>
   </si>
   <si>
     <t>18159.35</t>
   </si>
   <si>
-    <t>2023-01-03 00:00:00</t>
-  </si>
-  <si>
     <t>810,29</t>
   </si>
   <si>
     <t>4861.74</t>
   </si>
   <si>
-    <t>01/06/2023</t>
-  </si>
-  <si>
     <t>R$ 827.4</t>
   </si>
   <si>
     <t>1654.8</t>
   </si>
   <si>
-    <t>27/05/2023</t>
-  </si>
-  <si>
     <t>20 unidades</t>
   </si>
   <si>
@@ -906,13 +557,7 @@
     <t>4587,28</t>
   </si>
   <si>
-    <t>2023-06-03</t>
-  </si>
-  <si>
     <t>22540.76</t>
-  </si>
-  <si>
-    <t>2023-08-16 00:00:00</t>
   </si>
   <si>
     <t>26341.62</t>
@@ -922,8 +567,25 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="167" formatCode="&quot;R$&quot;\ #,##0.00"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -951,8 +613,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1233,385 +904,397 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G121"/>
+  <dimension ref="A1:I121"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.140625" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="18.140625" customWidth="1"/>
+    <col min="6" max="6" width="21" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" customWidth="1"/>
+    <col min="9" max="9" width="11.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>45141</v>
+      </c>
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>9</v>
-      </c>
-      <c r="D2" t="s">
-        <v>10</v>
       </c>
       <c r="E2">
         <v>14</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="3">
         <v>3139.25</v>
       </c>
       <c r="G2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="1"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>45041</v>
+      </c>
+      <c r="B3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="C3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
         <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
       </c>
       <c r="E3">
         <v>13</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="3">
         <v>345.37</v>
       </c>
       <c r="G3">
         <v>6216.66</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>16</v>
+      <c r="I3" s="1"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>44966</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E4">
         <v>15</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="3">
         <v>825.2</v>
       </c>
       <c r="G4">
         <v>2475.6</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>19</v>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>45111</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E5">
         <v>7</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="3">
         <v>2873.97</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>22</v>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>44943</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E6">
         <v>7</v>
       </c>
-      <c r="F6" t="s">
-        <v>25</v>
+      <c r="F6" s="3">
+        <v>760.94</v>
       </c>
       <c r="G6">
         <v>8370.34</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>26</v>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>45288</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E7">
         <v>19</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="3">
         <v>380.24</v>
       </c>
       <c r="G7">
         <v>3422.16</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>28</v>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>45225</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E8" t="s">
-        <v>30</v>
-      </c>
-      <c r="F8" t="s">
-        <v>31</v>
+        <v>22</v>
+      </c>
+      <c r="F8" s="3">
+        <v>2465.4499999999998</v>
       </c>
       <c r="G8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>33</v>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>44933</v>
       </c>
       <c r="B9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" t="s">
         <v>24</v>
       </c>
-      <c r="E9" t="s">
-        <v>34</v>
-      </c>
-      <c r="F9" t="s">
-        <v>35</v>
+      <c r="F9" s="3">
+        <v>758.5</v>
       </c>
       <c r="G9">
         <v>1517</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>36</v>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>44997</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="D10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E10" t="s">
-        <v>38</v>
-      </c>
-      <c r="F10">
+        <v>26</v>
+      </c>
+      <c r="F10" s="3">
         <v>2166.89</v>
       </c>
-      <c r="G10" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>40</v>
+      <c r="G10" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>45276</v>
       </c>
       <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" t="s">
         <v>20</v>
       </c>
-      <c r="C11" t="s">
-        <v>27</v>
-      </c>
       <c r="D11" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E11" t="s">
-        <v>42</v>
-      </c>
-      <c r="F11" t="s">
-        <v>43</v>
+        <v>29</v>
+      </c>
+      <c r="F11" s="3">
+        <v>2649.97</v>
       </c>
       <c r="G11">
         <v>15899.82</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>44</v>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>44938</v>
       </c>
       <c r="B12" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="D12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E12" t="s">
-        <v>46</v>
-      </c>
-      <c r="F12" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>48</v>
+        <v>31</v>
+      </c>
+      <c r="F12" s="3">
+        <v>1855.07</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>44971</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D13" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E13" t="s">
-        <v>50</v>
-      </c>
-      <c r="F13" t="s">
-        <v>51</v>
+        <v>33</v>
+      </c>
+      <c r="F13" s="3">
+        <v>4836.45</v>
       </c>
       <c r="G13" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>53</v>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>45131</v>
       </c>
       <c r="B14" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D14" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E14" t="s">
-        <v>54</v>
-      </c>
-      <c r="F14" t="s">
-        <v>55</v>
+        <v>35</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>36</v>
       </c>
       <c r="G14" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>57</v>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>44937</v>
       </c>
       <c r="B15" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C15" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D15" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E15">
         <v>11</v>
       </c>
-      <c r="F15" t="s">
-        <v>58</v>
+      <c r="F15" s="3">
+        <v>4133.8500000000004</v>
       </c>
       <c r="G15" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>45111</v>
+      </c>
+      <c r="B16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" t="s">
         <v>19</v>
-      </c>
-      <c r="B16" t="s">
-        <v>20</v>
-      </c>
-      <c r="C16" t="s">
-        <v>60</v>
-      </c>
-      <c r="D16" t="s">
-        <v>24</v>
       </c>
       <c r="E16">
         <v>10</v>
       </c>
-      <c r="F16" t="s">
-        <v>61</v>
+      <c r="F16" s="3" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>62</v>
+      <c r="A17" s="1">
+        <v>45037</v>
       </c>
       <c r="B17" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C17" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D17" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E17">
         <v>17</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="3">
         <v>4668.8900000000003</v>
       </c>
       <c r="G17">
@@ -1619,553 +1302,553 @@
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>63</v>
+      <c r="A18" s="1">
+        <v>45188</v>
       </c>
       <c r="B18" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C18" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D18" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E18">
         <v>8</v>
       </c>
-      <c r="F18" t="s">
-        <v>64</v>
+      <c r="F18" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="G18" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>66</v>
+      <c r="A19" s="1">
+        <v>45177</v>
       </c>
       <c r="B19" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C19" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="D19" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E19" t="s">
-        <v>67</v>
-      </c>
-      <c r="F19" t="s">
-        <v>68</v>
+        <v>43</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>69</v>
+      <c r="A20" s="1">
+        <v>45036</v>
       </c>
       <c r="B20" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C20" t="s">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="D20" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E20" t="s">
-        <v>71</v>
-      </c>
-      <c r="F20" t="s">
-        <v>72</v>
+        <v>46</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>47</v>
       </c>
       <c r="G20">
         <v>1152.54</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>73</v>
+      <c r="A21" s="1">
+        <v>45114</v>
       </c>
       <c r="B21" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C21" t="s">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="D21" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E21" t="s">
-        <v>74</v>
-      </c>
-      <c r="F21" t="s">
-        <v>75</v>
+        <v>48</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>76</v>
+      <c r="A22" s="1">
+        <v>44979</v>
       </c>
       <c r="B22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" t="s">
+        <v>50</v>
+      </c>
+      <c r="D22" t="s">
+        <v>28</v>
+      </c>
+      <c r="E22" t="s">
+        <v>51</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G22" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>45280</v>
+      </c>
+      <c r="B23" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" t="s">
         <v>20</v>
       </c>
-      <c r="C22" t="s">
-        <v>77</v>
-      </c>
-      <c r="D22" t="s">
-        <v>41</v>
-      </c>
-      <c r="E22" t="s">
-        <v>78</v>
-      </c>
-      <c r="F22" t="s">
-        <v>79</v>
-      </c>
-      <c r="G22" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>81</v>
-      </c>
-      <c r="B23" t="s">
-        <v>82</v>
-      </c>
-      <c r="C23" t="s">
-        <v>27</v>
-      </c>
       <c r="D23" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E23" t="s">
-        <v>83</v>
-      </c>
-      <c r="F23" t="s">
-        <v>84</v>
+        <v>55</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>56</v>
       </c>
       <c r="G23" t="s">
-        <v>85</v>
+        <v>57</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>86</v>
+      <c r="A24" s="1">
+        <v>45065</v>
       </c>
       <c r="B24" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C24" t="s">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="D24" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E24" t="s">
-        <v>42</v>
-      </c>
-      <c r="F24" t="s">
-        <v>88</v>
+        <v>29</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>89</v>
+      <c r="A25" s="1">
+        <v>45091</v>
       </c>
       <c r="B25" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C25" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D25" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E25" t="s">
-        <v>90</v>
-      </c>
-      <c r="F25" t="s">
-        <v>91</v>
+        <v>60</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="G25">
         <v>27011.79</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>92</v>
+      <c r="A26" s="1">
+        <v>45121</v>
       </c>
       <c r="B26" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C26" t="s">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="D26" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E26" t="s">
-        <v>93</v>
-      </c>
-      <c r="F26" t="s">
-        <v>94</v>
+        <v>62</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>63</v>
       </c>
       <c r="G26" t="s">
-        <v>95</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>96</v>
+      <c r="A27" s="1">
+        <v>45205</v>
       </c>
       <c r="B27" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C27" t="s">
-        <v>97</v>
+        <v>65</v>
       </c>
       <c r="D27" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E27" t="s">
-        <v>98</v>
-      </c>
-      <c r="F27" t="s">
-        <v>99</v>
+        <v>66</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>67</v>
       </c>
       <c r="G27">
         <v>15228.5</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>100</v>
+      <c r="A28" s="1">
+        <v>44967</v>
       </c>
       <c r="B28" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C28" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="D28" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" t="s">
+        <v>55</v>
+      </c>
+      <c r="F28" s="3">
+        <v>979.88</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>45195</v>
+      </c>
+      <c r="B29" t="s">
+        <v>54</v>
+      </c>
+      <c r="C29" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" t="s">
+        <v>28</v>
+      </c>
+      <c r="E29" t="s">
+        <v>68</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="G29" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>45101</v>
+      </c>
+      <c r="B30" t="s">
         <v>18</v>
       </c>
-      <c r="E28" t="s">
-        <v>83</v>
-      </c>
-      <c r="F28">
-        <v>979.88</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>101</v>
-      </c>
-      <c r="B29" t="s">
-        <v>82</v>
-      </c>
-      <c r="C29" t="s">
-        <v>14</v>
-      </c>
-      <c r="D29" t="s">
-        <v>41</v>
-      </c>
-      <c r="E29" t="s">
-        <v>102</v>
-      </c>
-      <c r="F29" t="s">
-        <v>103</v>
-      </c>
-      <c r="G29" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>105</v>
-      </c>
-      <c r="B30" t="s">
-        <v>23</v>
-      </c>
       <c r="C30" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D30" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E30">
         <v>8</v>
       </c>
-      <c r="F30" t="s">
-        <v>106</v>
+      <c r="F30" s="3" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>107</v>
+      <c r="A31" s="1">
+        <v>45012</v>
       </c>
       <c r="B31" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C31" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D31" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E31">
         <v>12</v>
       </c>
-      <c r="F31" t="s">
-        <v>108</v>
+      <c r="F31" s="3" t="s">
+        <v>72</v>
       </c>
       <c r="G31">
         <v>19460.14</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>109</v>
+      <c r="A32" s="1">
+        <v>45072</v>
       </c>
       <c r="B32" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C32" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D32" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E32" t="s">
+        <v>48</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="G32" t="s">
         <v>74</v>
       </c>
-      <c r="F32" t="s">
-        <v>110</v>
-      </c>
-      <c r="G32" t="s">
-        <v>111</v>
-      </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>112</v>
+      <c r="A33" s="1">
+        <v>45106</v>
       </c>
       <c r="B33" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C33" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D33" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E33">
         <v>18</v>
       </c>
-      <c r="F33">
+      <c r="F33" s="3">
         <v>4896.72</v>
       </c>
       <c r="G33" t="s">
-        <v>113</v>
+        <v>75</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>114</v>
+      <c r="A34" s="1">
+        <v>44973</v>
       </c>
       <c r="B34" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C34" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="D34" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E34">
         <v>4</v>
       </c>
-      <c r="F34" t="s">
-        <v>115</v>
+      <c r="F34" s="3" t="s">
+        <v>76</v>
       </c>
       <c r="G34">
         <v>50350.3</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>89</v>
+      <c r="A35" s="1">
+        <v>45091</v>
       </c>
       <c r="B35" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C35" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="D35" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E35">
         <v>10</v>
       </c>
-      <c r="F35" t="s">
-        <v>116</v>
+      <c r="F35" s="3" t="s">
+        <v>77</v>
       </c>
       <c r="G35">
         <v>14016.9</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>117</v>
+      <c r="A36" s="1">
+        <v>45068</v>
       </c>
       <c r="B36" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C36" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="D36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E36" t="s">
-        <v>34</v>
-      </c>
-      <c r="F36" t="s">
-        <v>118</v>
+        <v>24</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>78</v>
       </c>
       <c r="G36">
         <v>7245.21</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>119</v>
+      <c r="A37" s="1">
+        <v>45091</v>
       </c>
       <c r="B37" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="C37" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D37" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E37">
         <v>10</v>
       </c>
-      <c r="F37">
+      <c r="F37" s="3">
         <v>4776.49</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>120</v>
+      <c r="A38" s="1">
+        <v>44954</v>
       </c>
       <c r="B38" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C38" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
       <c r="D38" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E38" t="s">
-        <v>38</v>
-      </c>
-      <c r="F38" t="s">
-        <v>122</v>
+        <v>26</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>80</v>
       </c>
       <c r="G38" t="s">
-        <v>123</v>
+        <v>81</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>124</v>
+      <c r="A39" s="1">
+        <v>45020</v>
       </c>
       <c r="B39" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="C39" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D39" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E39">
         <v>13</v>
       </c>
-      <c r="F39">
+      <c r="F39" s="3">
         <v>423.3</v>
       </c>
       <c r="G39" t="s">
-        <v>125</v>
+        <v>82</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>126</v>
+      <c r="A40" s="1">
+        <v>45218</v>
       </c>
       <c r="B40" t="s">
+        <v>11</v>
+      </c>
+      <c r="C40" t="s">
+        <v>30</v>
+      </c>
+      <c r="D40" t="s">
         <v>13</v>
-      </c>
-      <c r="C40" t="s">
-        <v>45</v>
-      </c>
-      <c r="D40" t="s">
-        <v>15</v>
       </c>
       <c r="E40">
         <v>6</v>
       </c>
-      <c r="F40" t="s">
-        <v>127</v>
+      <c r="F40" s="3" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>128</v>
+      <c r="A41" s="1">
+        <v>45226</v>
       </c>
       <c r="B41" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C41" t="s">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="D41" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E41">
         <v>14</v>
       </c>
-      <c r="F41" t="s">
-        <v>129</v>
+      <c r="F41" s="3" t="s">
+        <v>84</v>
       </c>
       <c r="G41" t="s">
-        <v>130</v>
+        <v>85</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>131</v>
+      <c r="A42" s="1">
+        <v>45152</v>
       </c>
       <c r="B42" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C42" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D42" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E42">
         <v>11</v>
       </c>
-      <c r="F42">
+      <c r="F42" s="3">
         <v>1649.02</v>
       </c>
       <c r="G42">
@@ -2173,197 +1856,197 @@
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>132</v>
+      <c r="A43" s="1">
+        <v>45069</v>
       </c>
       <c r="B43" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C43" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="D43" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E43">
         <v>13</v>
       </c>
-      <c r="F43" t="s">
-        <v>133</v>
+      <c r="F43" s="3" t="s">
+        <v>86</v>
       </c>
       <c r="G43">
         <v>40814.730000000003</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>134</v>
+      <c r="A44" s="1">
+        <v>45027</v>
       </c>
       <c r="B44" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C44" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D44" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E44" t="s">
-        <v>50</v>
-      </c>
-      <c r="F44" t="s">
-        <v>135</v>
+        <v>33</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>136</v>
+      <c r="A45" s="1">
+        <v>44999</v>
       </c>
       <c r="B45" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C45" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D45" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E45">
         <v>17</v>
       </c>
-      <c r="F45">
+      <c r="F45" s="3">
         <v>4697.54</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>137</v>
+      <c r="A46" s="1">
+        <v>45132</v>
       </c>
       <c r="B46" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C46" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D46" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E46">
         <v>7</v>
       </c>
-      <c r="F46" t="s">
-        <v>138</v>
+      <c r="F46" s="3" t="s">
+        <v>88</v>
       </c>
       <c r="G46" t="s">
-        <v>139</v>
+        <v>89</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>140</v>
+      <c r="A47" s="1">
+        <v>45219</v>
       </c>
       <c r="B47" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="C47" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="D47" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E47">
         <v>2</v>
       </c>
-      <c r="F47" t="s">
-        <v>141</v>
+      <c r="F47" s="3" t="s">
+        <v>90</v>
       </c>
       <c r="G47">
         <v>1650.69</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>142</v>
+      <c r="A48" s="1">
+        <v>45273</v>
       </c>
       <c r="B48" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C48" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="D48" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E48">
         <v>16</v>
       </c>
-      <c r="F48" t="s">
-        <v>143</v>
+      <c r="F48" s="3" t="s">
+        <v>91</v>
       </c>
       <c r="G48">
         <v>5367.48</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>144</v>
+      <c r="A49" s="1">
+        <v>45140</v>
       </c>
       <c r="B49" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C49" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D49" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E49">
         <v>18</v>
       </c>
-      <c r="F49" t="s">
-        <v>145</v>
+      <c r="F49" s="3" t="s">
+        <v>92</v>
       </c>
       <c r="G49">
         <v>94270.399999999994</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>146</v>
+      <c r="A50" s="1">
+        <v>45207</v>
       </c>
       <c r="B50" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C50" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="D50" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E50">
         <v>16</v>
       </c>
-      <c r="F50" t="s">
-        <v>147</v>
+      <c r="F50" s="3" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>148</v>
+      <c r="A51" s="1">
+        <v>44975</v>
       </c>
       <c r="B51" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C51" t="s">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="D51" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E51">
         <v>10</v>
       </c>
-      <c r="F51">
+      <c r="F51" s="3">
         <v>3936.93</v>
       </c>
       <c r="G51">
@@ -2371,220 +2054,220 @@
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>149</v>
+      <c r="A52" s="1">
+        <v>44977</v>
       </c>
       <c r="B52" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C52" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="D52" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E52" t="s">
-        <v>71</v>
-      </c>
-      <c r="F52">
+        <v>46</v>
+      </c>
+      <c r="F52" s="3">
         <v>4087.23</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>150</v>
+      <c r="A53" s="1">
+        <v>45280</v>
       </c>
       <c r="B53" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C53" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="D53" t="s">
+        <v>15</v>
+      </c>
+      <c r="E53" t="s">
+        <v>29</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
+        <v>45274</v>
+      </c>
+      <c r="B54" t="s">
         <v>18</v>
       </c>
-      <c r="E53" t="s">
-        <v>42</v>
-      </c>
-      <c r="F53" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>152</v>
-      </c>
-      <c r="B54" t="s">
-        <v>23</v>
-      </c>
       <c r="C54" t="s">
-        <v>97</v>
+        <v>65</v>
       </c>
       <c r="D54" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E54">
         <v>17</v>
       </c>
-      <c r="F54" t="s">
-        <v>153</v>
+      <c r="F54" s="3" t="s">
+        <v>95</v>
       </c>
       <c r="G54">
         <v>2849.38</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>154</v>
+      <c r="A55" s="1">
+        <v>45182</v>
       </c>
       <c r="B55" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C55" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D55" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E55">
         <v>8</v>
       </c>
-      <c r="F55" t="s">
-        <v>155</v>
+      <c r="F55" s="3" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>156</v>
+      <c r="A56" s="1">
+        <v>45194</v>
       </c>
       <c r="B56" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C56" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D56" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E56" t="s">
-        <v>50</v>
-      </c>
-      <c r="F56" t="s">
-        <v>157</v>
+        <v>33</v>
+      </c>
+      <c r="F56" s="3" t="s">
+        <v>97</v>
       </c>
       <c r="G56">
         <v>1355.25</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>158</v>
+      <c r="A57" s="1">
+        <v>45271</v>
       </c>
       <c r="B57" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C57" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
       <c r="D57" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E57">
         <v>8</v>
       </c>
-      <c r="F57" t="s">
-        <v>159</v>
+      <c r="F57" s="3" t="s">
+        <v>98</v>
       </c>
       <c r="G57">
         <v>35404.199999999997</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>160</v>
+      <c r="A58" s="1">
+        <v>45146</v>
       </c>
       <c r="B58" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="C58" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="D58" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E58">
         <v>16</v>
       </c>
-      <c r="F58">
+      <c r="F58" s="3">
         <v>1211.28</v>
       </c>
       <c r="G58" t="s">
-        <v>161</v>
+        <v>99</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>162</v>
+      <c r="A59" s="1">
+        <v>45264</v>
       </c>
       <c r="B59" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C59" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="D59" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E59">
         <v>12</v>
       </c>
-      <c r="F59">
+      <c r="F59" s="3">
         <v>1417.08</v>
       </c>
       <c r="G59" t="s">
-        <v>163</v>
+        <v>100</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>164</v>
+      <c r="A60" s="1">
+        <v>45161</v>
       </c>
       <c r="B60" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C60" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
       <c r="D60" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E60">
         <v>16</v>
       </c>
-      <c r="F60" t="s">
-        <v>165</v>
+      <c r="F60" s="3" t="s">
+        <v>101</v>
       </c>
       <c r="G60" t="s">
-        <v>166</v>
+        <v>102</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>167</v>
+      <c r="A61" s="1">
+        <v>45140</v>
       </c>
       <c r="B61" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C61" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="D61" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E61" t="s">
-        <v>90</v>
-      </c>
-      <c r="F61">
+        <v>60</v>
+      </c>
+      <c r="F61" s="3">
         <v>775.3</v>
       </c>
       <c r="G61">
@@ -2592,659 +2275,659 @@
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>168</v>
+      <c r="A62" s="1">
+        <v>45169</v>
       </c>
       <c r="B62" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C62" t="s">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="D62" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E62" t="s">
-        <v>46</v>
-      </c>
-      <c r="F62" t="s">
-        <v>169</v>
+        <v>31</v>
+      </c>
+      <c r="F62" s="3" t="s">
+        <v>103</v>
       </c>
       <c r="G62" t="s">
-        <v>170</v>
+        <v>104</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>171</v>
+      <c r="A63" s="1">
+        <v>45218</v>
       </c>
       <c r="B63" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C63" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D63" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E63" t="s">
-        <v>93</v>
-      </c>
-      <c r="F63">
+        <v>62</v>
+      </c>
+      <c r="F63" s="3">
         <v>2388.29</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>172</v>
+      <c r="A64" s="1">
+        <v>45082</v>
       </c>
       <c r="B64" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C64" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="D64" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E64">
         <v>10</v>
       </c>
-      <c r="F64">
+      <c r="F64" s="3">
         <v>3624.07</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>173</v>
+      <c r="A65" s="1">
+        <v>45155</v>
       </c>
       <c r="B65" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C65" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D65" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E65">
         <v>20</v>
       </c>
-      <c r="F65" t="s">
-        <v>174</v>
+      <c r="F65" s="3" t="s">
+        <v>105</v>
       </c>
       <c r="G65">
         <v>4847.9399999999996</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>175</v>
+      <c r="A66" s="1">
+        <v>45047</v>
       </c>
       <c r="B66" t="s">
+        <v>11</v>
+      </c>
+      <c r="C66" t="s">
+        <v>12</v>
+      </c>
+      <c r="D66" t="s">
         <v>13</v>
-      </c>
-      <c r="C66" t="s">
-        <v>14</v>
-      </c>
-      <c r="D66" t="s">
-        <v>15</v>
       </c>
       <c r="E66">
         <v>7</v>
       </c>
-      <c r="F66" t="s">
-        <v>176</v>
+      <c r="F66" s="3" t="s">
+        <v>106</v>
       </c>
       <c r="G66">
         <v>41961.599999999999</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>177</v>
+      <c r="A67" s="1">
+        <v>45291</v>
       </c>
       <c r="B67" t="s">
+        <v>7</v>
+      </c>
+      <c r="C67" t="s">
+        <v>25</v>
+      </c>
+      <c r="D67" t="s">
+        <v>28</v>
+      </c>
+      <c r="E67" t="s">
+        <v>51</v>
+      </c>
+      <c r="F67" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A68" s="1">
+        <v>44959</v>
+      </c>
+      <c r="B68" t="s">
+        <v>16</v>
+      </c>
+      <c r="C68" t="s">
         <v>8</v>
       </c>
-      <c r="C67" t="s">
-        <v>37</v>
-      </c>
-      <c r="D67" t="s">
-        <v>41</v>
-      </c>
-      <c r="E67" t="s">
-        <v>78</v>
-      </c>
-      <c r="F67" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>179</v>
-      </c>
-      <c r="B68" t="s">
-        <v>20</v>
-      </c>
-      <c r="C68" t="s">
-        <v>9</v>
-      </c>
       <c r="D68" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E68" t="s">
-        <v>180</v>
-      </c>
-      <c r="F68" t="s">
-        <v>181</v>
+        <v>108</v>
+      </c>
+      <c r="F68" s="3" t="s">
+        <v>109</v>
       </c>
       <c r="G68">
         <v>42995.7</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>182</v>
+      <c r="A69" s="1">
+        <v>45128</v>
       </c>
       <c r="B69" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="C69" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D69" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E69">
         <v>20</v>
       </c>
-      <c r="F69" t="s">
-        <v>183</v>
+      <c r="F69" s="3" t="s">
+        <v>110</v>
       </c>
       <c r="G69" t="s">
-        <v>184</v>
+        <v>111</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>185</v>
+      <c r="A70" s="1">
+        <v>45187</v>
       </c>
       <c r="B70" t="s">
+        <v>11</v>
+      </c>
+      <c r="C70" t="s">
+        <v>20</v>
+      </c>
+      <c r="D70" t="s">
+        <v>15</v>
+      </c>
+      <c r="E70" t="s">
+        <v>60</v>
+      </c>
+      <c r="F70" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A71" s="1">
+        <v>45196</v>
+      </c>
+      <c r="B71" t="s">
+        <v>16</v>
+      </c>
+      <c r="C71" t="s">
+        <v>17</v>
+      </c>
+      <c r="D71" t="s">
         <v>13</v>
-      </c>
-      <c r="C70" t="s">
-        <v>27</v>
-      </c>
-      <c r="D70" t="s">
-        <v>18</v>
-      </c>
-      <c r="E70" t="s">
-        <v>90</v>
-      </c>
-      <c r="F70" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>187</v>
-      </c>
-      <c r="B71" t="s">
-        <v>20</v>
-      </c>
-      <c r="C71" t="s">
-        <v>21</v>
-      </c>
-      <c r="D71" t="s">
-        <v>15</v>
       </c>
       <c r="E71">
         <v>8</v>
       </c>
-      <c r="F71" t="s">
-        <v>188</v>
+      <c r="F71" s="3" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>189</v>
+      <c r="A72" s="1">
+        <v>45062</v>
       </c>
       <c r="B72" t="s">
+        <v>16</v>
+      </c>
+      <c r="C72" t="s">
         <v>20</v>
       </c>
-      <c r="C72" t="s">
-        <v>27</v>
-      </c>
       <c r="D72" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E72" t="s">
-        <v>83</v>
-      </c>
-      <c r="F72" t="s">
-        <v>190</v>
+        <v>55</v>
+      </c>
+      <c r="F72" s="3" t="s">
+        <v>114</v>
       </c>
       <c r="G72">
         <v>27462.82</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>191</v>
+      <c r="A73" s="1">
+        <v>45286</v>
       </c>
       <c r="B73" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="C73" t="s">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="D73" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E73">
         <v>1</v>
       </c>
-      <c r="F73" t="s">
-        <v>192</v>
+      <c r="F73" s="3" t="s">
+        <v>115</v>
       </c>
       <c r="G73" t="s">
-        <v>193</v>
+        <v>116</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>194</v>
+      <c r="A74" s="1">
+        <v>45169</v>
       </c>
       <c r="B74" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C74" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
       <c r="D74" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E74">
         <v>11</v>
       </c>
-      <c r="F74" t="s">
-        <v>195</v>
+      <c r="F74" s="3" t="s">
+        <v>117</v>
       </c>
       <c r="G74" t="s">
-        <v>196</v>
+        <v>118</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>197</v>
+      <c r="A75" s="1">
+        <v>44944</v>
       </c>
       <c r="B75" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C75" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D75" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E75">
         <v>14</v>
       </c>
-      <c r="F75" t="s">
-        <v>198</v>
+      <c r="F75" s="3" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>199</v>
+      <c r="A76" s="1">
+        <v>45211</v>
       </c>
       <c r="B76" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C76" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D76" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E76">
         <v>5</v>
       </c>
-      <c r="F76" t="s">
-        <v>200</v>
+      <c r="F76" s="3" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>201</v>
+      <c r="A77" s="1">
+        <v>45070</v>
       </c>
       <c r="B77" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C77" t="s">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="D77" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E77">
         <v>9</v>
       </c>
-      <c r="F77" t="s">
-        <v>202</v>
+      <c r="F77" s="3" t="s">
+        <v>121</v>
       </c>
       <c r="G77">
         <v>591.94000000000005</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>203</v>
+      <c r="A78" s="1">
+        <v>45266</v>
       </c>
       <c r="B78" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C78" t="s">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="D78" t="s">
+        <v>13</v>
+      </c>
+      <c r="E78" t="s">
+        <v>24</v>
+      </c>
+      <c r="F78" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="G78" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A79" s="1">
+        <v>45117</v>
+      </c>
+      <c r="B79" t="s">
+        <v>18</v>
+      </c>
+      <c r="C79" t="s">
+        <v>30</v>
+      </c>
+      <c r="D79" t="s">
         <v>15</v>
       </c>
-      <c r="E78" t="s">
-        <v>34</v>
-      </c>
-      <c r="F78" t="s">
-        <v>204</v>
-      </c>
-      <c r="G78" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>206</v>
-      </c>
-      <c r="B79" t="s">
-        <v>23</v>
-      </c>
-      <c r="C79" t="s">
-        <v>45</v>
-      </c>
-      <c r="D79" t="s">
-        <v>18</v>
-      </c>
       <c r="E79" t="s">
-        <v>30</v>
-      </c>
-      <c r="F79">
+        <v>22</v>
+      </c>
+      <c r="F79" s="3">
         <v>2139.87</v>
       </c>
       <c r="G79" t="s">
-        <v>207</v>
+        <v>124</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
-        <v>208</v>
+      <c r="A80" s="1">
+        <v>45016</v>
       </c>
       <c r="B80" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C80" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D80" t="s">
+        <v>13</v>
+      </c>
+      <c r="E80" t="s">
+        <v>125</v>
+      </c>
+      <c r="F80" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A81" s="1">
+        <v>45086</v>
+      </c>
+      <c r="B81" t="s">
+        <v>16</v>
+      </c>
+      <c r="C81" t="s">
+        <v>14</v>
+      </c>
+      <c r="D81" t="s">
         <v>15</v>
-      </c>
-      <c r="E80" t="s">
-        <v>209</v>
-      </c>
-      <c r="F80" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>211</v>
-      </c>
-      <c r="B81" t="s">
-        <v>20</v>
-      </c>
-      <c r="C81" t="s">
-        <v>17</v>
-      </c>
-      <c r="D81" t="s">
-        <v>18</v>
       </c>
       <c r="E81">
         <v>3</v>
       </c>
-      <c r="F81" t="s">
-        <v>212</v>
+      <c r="F81" s="3" t="s">
+        <v>127</v>
       </c>
       <c r="G81" t="s">
-        <v>213</v>
+        <v>128</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>214</v>
+      <c r="A82" s="1">
+        <v>45251</v>
       </c>
       <c r="B82" t="s">
+        <v>7</v>
+      </c>
+      <c r="C82" t="s">
         <v>8</v>
       </c>
-      <c r="C82" t="s">
-        <v>9</v>
-      </c>
       <c r="D82" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E82" t="s">
-        <v>209</v>
-      </c>
-      <c r="F82" t="s">
-        <v>215</v>
+        <v>125</v>
+      </c>
+      <c r="F82" s="3" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>216</v>
+      <c r="A83" s="1">
+        <v>45058</v>
       </c>
       <c r="B83" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C83" t="s">
-        <v>97</v>
+        <v>65</v>
       </c>
       <c r="D83" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E83">
         <v>7</v>
       </c>
-      <c r="F83" t="s">
-        <v>217</v>
+      <c r="F83" s="3" t="s">
+        <v>130</v>
       </c>
       <c r="G83">
         <v>63043.9</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>218</v>
+      <c r="A84" s="1">
+        <v>44947</v>
       </c>
       <c r="B84" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C84" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D84" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E84" t="s">
-        <v>74</v>
-      </c>
-      <c r="F84" t="s">
-        <v>219</v>
+        <v>48</v>
+      </c>
+      <c r="F84" s="3" t="s">
+        <v>131</v>
       </c>
       <c r="G84">
         <v>45948.27</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>220</v>
+      <c r="A85" s="1">
+        <v>44980</v>
       </c>
       <c r="B85" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C85" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="D85" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E85">
         <v>14</v>
       </c>
-      <c r="F85">
+      <c r="F85" s="3">
         <v>2679.53</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>221</v>
+      <c r="A86" s="1">
+        <v>45040</v>
       </c>
       <c r="B86" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C86" t="s">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="D86" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E86">
         <v>1</v>
       </c>
-      <c r="F86" t="s">
-        <v>222</v>
+      <c r="F86" s="3" t="s">
+        <v>132</v>
       </c>
       <c r="G86" t="s">
-        <v>223</v>
+        <v>133</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>224</v>
+      <c r="A87" s="1">
+        <v>45182</v>
       </c>
       <c r="B87" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C87" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="D87" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E87" t="s">
-        <v>54</v>
-      </c>
-      <c r="F87" t="s">
-        <v>225</v>
+        <v>35</v>
+      </c>
+      <c r="F87" s="3" t="s">
+        <v>134</v>
       </c>
       <c r="G87">
         <v>1559.04</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>226</v>
+      <c r="A88" s="1">
+        <v>44981</v>
       </c>
       <c r="B88" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C88" t="s">
-        <v>97</v>
+        <v>65</v>
       </c>
       <c r="D88" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E88" t="s">
-        <v>46</v>
-      </c>
-      <c r="F88" t="s">
-        <v>227</v>
+        <v>31</v>
+      </c>
+      <c r="F88" s="3" t="s">
+        <v>135</v>
       </c>
       <c r="G88">
         <v>2472.09</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
-        <v>228</v>
+      <c r="A89" s="1">
+        <v>45213</v>
       </c>
       <c r="B89" t="s">
+        <v>11</v>
+      </c>
+      <c r="C89" t="s">
+        <v>30</v>
+      </c>
+      <c r="D89" t="s">
         <v>13</v>
       </c>
-      <c r="C89" t="s">
+      <c r="E89" t="s">
+        <v>35</v>
+      </c>
+      <c r="F89" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="G89" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A90" s="1">
+        <v>45133</v>
+      </c>
+      <c r="B90" t="s">
+        <v>54</v>
+      </c>
+      <c r="C90" t="s">
         <v>45</v>
       </c>
-      <c r="D89" t="s">
+      <c r="D90" t="s">
         <v>15</v>
-      </c>
-      <c r="E89" t="s">
-        <v>54</v>
-      </c>
-      <c r="F89" t="s">
-        <v>229</v>
-      </c>
-      <c r="G89" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>231</v>
-      </c>
-      <c r="B90" t="s">
-        <v>82</v>
-      </c>
-      <c r="C90" t="s">
-        <v>70</v>
-      </c>
-      <c r="D90" t="s">
-        <v>18</v>
       </c>
       <c r="E90">
         <v>3</v>
       </c>
-      <c r="F90" t="s">
-        <v>232</v>
+      <c r="F90" s="3" t="s">
+        <v>138</v>
       </c>
       <c r="G90" t="s">
-        <v>233</v>
+        <v>139</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>234</v>
+      <c r="A91" s="1">
+        <v>45133</v>
       </c>
       <c r="B91" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C91" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D91" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E91" t="s">
-        <v>34</v>
-      </c>
-      <c r="F91">
+        <v>24</v>
+      </c>
+      <c r="F91" s="3">
         <v>3418.73</v>
       </c>
       <c r="G91">
@@ -3252,332 +2935,332 @@
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>235</v>
+      <c r="A92" s="1">
+        <v>45029</v>
       </c>
       <c r="B92" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C92" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="D92" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E92" t="s">
-        <v>83</v>
-      </c>
-      <c r="F92" t="s">
-        <v>236</v>
+        <v>55</v>
+      </c>
+      <c r="F92" s="3" t="s">
+        <v>140</v>
       </c>
       <c r="G92" t="s">
-        <v>237</v>
+        <v>141</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
-        <v>44</v>
+      <c r="A93" s="1">
+        <v>45261</v>
       </c>
       <c r="B93" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C93" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D93" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E93">
         <v>5</v>
       </c>
-      <c r="F93" t="s">
-        <v>238</v>
+      <c r="F93" s="3" t="s">
+        <v>142</v>
       </c>
       <c r="G93" t="s">
-        <v>239</v>
+        <v>143</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>240</v>
+      <c r="A94" s="1">
+        <v>45248</v>
       </c>
       <c r="B94" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C94" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="D94" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E94" t="s">
-        <v>180</v>
-      </c>
-      <c r="F94" t="s">
-        <v>241</v>
+        <v>108</v>
+      </c>
+      <c r="F94" s="3" t="s">
+        <v>144</v>
       </c>
       <c r="G94">
         <v>23119.88</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>242</v>
+      <c r="A95" s="1">
+        <v>45093</v>
       </c>
       <c r="B95" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C95" t="s">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="D95" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E95">
         <v>20</v>
       </c>
-      <c r="F95" t="s">
-        <v>243</v>
+      <c r="F95" s="3" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>244</v>
+      <c r="A96" s="1">
+        <v>45081</v>
       </c>
       <c r="B96" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C96" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D96" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E96" t="s">
-        <v>50</v>
-      </c>
-      <c r="F96" t="s">
-        <v>245</v>
+        <v>33</v>
+      </c>
+      <c r="F96" s="3" t="s">
+        <v>146</v>
       </c>
       <c r="G96">
         <v>31034.99</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>246</v>
+      <c r="A97" s="1">
+        <v>44959</v>
       </c>
       <c r="B97" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="C97" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
       <c r="D97" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E97">
         <v>2</v>
       </c>
-      <c r="F97">
+      <c r="F97" s="3">
         <v>1034.1099999999999</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>247</v>
+      <c r="A98" s="1">
+        <v>45097</v>
       </c>
       <c r="B98" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="C98" t="s">
+        <v>21</v>
+      </c>
+      <c r="D98" t="s">
+        <v>28</v>
+      </c>
+      <c r="E98" t="s">
         <v>29</v>
       </c>
-      <c r="D98" t="s">
-        <v>41</v>
-      </c>
-      <c r="E98" t="s">
-        <v>42</v>
-      </c>
-      <c r="F98" t="s">
-        <v>248</v>
+      <c r="F98" s="3" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>249</v>
+      <c r="A99" s="1">
+        <v>45012</v>
       </c>
       <c r="B99" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="C99" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="D99" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E99" t="s">
-        <v>250</v>
-      </c>
-      <c r="F99">
+        <v>148</v>
+      </c>
+      <c r="F99" s="3">
         <v>3109.51</v>
       </c>
       <c r="G99" t="s">
-        <v>251</v>
+        <v>149</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>252</v>
+      <c r="A100" s="1">
+        <v>45253</v>
       </c>
       <c r="B100" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C100" t="s">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="D100" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E100">
         <v>4</v>
       </c>
-      <c r="F100">
+      <c r="F100" s="3">
         <v>1570.38</v>
       </c>
       <c r="G100" t="s">
-        <v>253</v>
+        <v>150</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>254</v>
+      <c r="A101" s="1">
+        <v>45175</v>
       </c>
       <c r="B101" t="s">
+        <v>11</v>
+      </c>
+      <c r="C101" t="s">
+        <v>25</v>
+      </c>
+      <c r="D101" t="s">
         <v>13</v>
       </c>
-      <c r="C101" t="s">
-        <v>37</v>
-      </c>
-      <c r="D101" t="s">
-        <v>15</v>
-      </c>
       <c r="E101" t="s">
-        <v>250</v>
-      </c>
-      <c r="F101" t="s">
-        <v>255</v>
+        <v>148</v>
+      </c>
+      <c r="F101" s="3" t="s">
+        <v>151</v>
       </c>
       <c r="G101" t="s">
-        <v>256</v>
+        <v>152</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
-        <v>257</v>
+      <c r="A102" s="1">
+        <v>45268</v>
       </c>
       <c r="B102" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C102" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D102" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E102" t="s">
-        <v>67</v>
-      </c>
-      <c r="F102" t="s">
-        <v>258</v>
+        <v>43</v>
+      </c>
+      <c r="F102" s="3" t="s">
+        <v>153</v>
       </c>
       <c r="G102">
         <v>19227.509999999998</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>203</v>
+      <c r="A103" s="1">
+        <v>45266</v>
       </c>
       <c r="B103" t="s">
+        <v>11</v>
+      </c>
+      <c r="C103" t="s">
+        <v>65</v>
+      </c>
+      <c r="D103" t="s">
         <v>13</v>
-      </c>
-      <c r="C103" t="s">
-        <v>97</v>
-      </c>
-      <c r="D103" t="s">
-        <v>15</v>
       </c>
       <c r="E103">
         <v>15</v>
       </c>
-      <c r="F103">
+      <c r="F103" s="3">
         <v>1886.49</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
-        <v>259</v>
+      <c r="A104" s="1">
+        <v>45145</v>
       </c>
       <c r="B104" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C104" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D104" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E104">
         <v>3</v>
       </c>
-      <c r="F104" t="s">
-        <v>260</v>
+      <c r="F104" s="3" t="s">
+        <v>154</v>
       </c>
       <c r="G104" t="s">
-        <v>261</v>
+        <v>155</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
-        <v>262</v>
+      <c r="A105" s="1">
+        <v>45250</v>
       </c>
       <c r="B105" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C105" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="D105" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E105">
         <v>2</v>
       </c>
-      <c r="F105" t="s">
-        <v>263</v>
+      <c r="F105" s="3" t="s">
+        <v>156</v>
       </c>
       <c r="G105" t="s">
-        <v>264</v>
+        <v>157</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
-        <v>265</v>
+      <c r="A106" s="1">
+        <v>45173</v>
       </c>
       <c r="B106" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C106" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D106" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E106" t="s">
-        <v>54</v>
-      </c>
-      <c r="F106">
+        <v>35</v>
+      </c>
+      <c r="F106" s="3">
         <v>3110.71</v>
       </c>
       <c r="G106">
@@ -3585,65 +3268,65 @@
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
-        <v>266</v>
+      <c r="A107" s="1">
+        <v>45234</v>
       </c>
       <c r="B107" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C107" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="D107" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E107">
         <v>17</v>
       </c>
-      <c r="F107" t="s">
-        <v>267</v>
+      <c r="F107" s="3" t="s">
+        <v>158</v>
       </c>
       <c r="G107" t="s">
-        <v>268</v>
+        <v>159</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
-        <v>269</v>
+      <c r="A108" s="1">
+        <v>45144</v>
       </c>
       <c r="B108" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="C108" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D108" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E108">
         <v>17</v>
       </c>
-      <c r="F108" t="s">
-        <v>270</v>
+      <c r="F108" s="3" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
-        <v>271</v>
+      <c r="A109" s="1">
+        <v>45228</v>
       </c>
       <c r="B109" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C109" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="D109" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E109" t="s">
-        <v>67</v>
-      </c>
-      <c r="F109">
+        <v>43</v>
+      </c>
+      <c r="F109" s="3">
         <v>1108.71</v>
       </c>
       <c r="G109">
@@ -3651,22 +3334,22 @@
       </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
-        <v>272</v>
+      <c r="A110" s="1">
+        <v>45284</v>
       </c>
       <c r="B110" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C110" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D110" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E110" t="s">
-        <v>54</v>
-      </c>
-      <c r="F110">
+        <v>35</v>
+      </c>
+      <c r="F110" s="3">
         <v>670.54</v>
       </c>
       <c r="G110">
@@ -3674,22 +3357,22 @@
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
-        <v>273</v>
+      <c r="A111" s="1">
+        <v>45250</v>
       </c>
       <c r="B111" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="C111" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D111" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E111" t="s">
-        <v>30</v>
-      </c>
-      <c r="F111">
+        <v>22</v>
+      </c>
+      <c r="F111" s="3">
         <v>702.91</v>
       </c>
       <c r="G111">
@@ -3697,233 +3380,235 @@
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
-        <v>274</v>
+      <c r="A112" s="1">
+        <v>44983</v>
       </c>
       <c r="B112" t="s">
+        <v>16</v>
+      </c>
+      <c r="C112" t="s">
         <v>20</v>
       </c>
-      <c r="C112" t="s">
-        <v>27</v>
-      </c>
       <c r="D112" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E112" t="s">
-        <v>83</v>
-      </c>
-      <c r="F112" t="s">
-        <v>275</v>
+        <v>55</v>
+      </c>
+      <c r="F112" s="3">
+        <v>1348.91</v>
       </c>
       <c r="G112">
         <v>25629.29</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
-        <v>276</v>
+      <c r="A113" s="1">
+        <v>45263</v>
       </c>
       <c r="B113" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C113" t="s">
+        <v>8</v>
+      </c>
+      <c r="D113" t="s">
+        <v>13</v>
+      </c>
+      <c r="E113" t="s">
+        <v>31</v>
+      </c>
+      <c r="F113" s="3">
+        <v>3218.22</v>
+      </c>
+      <c r="G113" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A114" s="1">
+        <v>44990</v>
+      </c>
+      <c r="B114" t="s">
+        <v>54</v>
+      </c>
+      <c r="C114" t="s">
+        <v>65</v>
+      </c>
+      <c r="D114" t="s">
+        <v>19</v>
+      </c>
+      <c r="E114" t="s">
+        <v>29</v>
+      </c>
+      <c r="F114" s="3">
+        <v>303.69</v>
+      </c>
+      <c r="G114" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A115" s="1">
+        <v>45207</v>
+      </c>
+      <c r="B115" t="s">
+        <v>16</v>
+      </c>
+      <c r="C115" t="s">
+        <v>32</v>
+      </c>
+      <c r="D115" t="s">
+        <v>15</v>
+      </c>
+      <c r="E115" t="s">
+        <v>55</v>
+      </c>
+      <c r="F115" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="G115" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A116" s="1">
+        <v>44986</v>
+      </c>
+      <c r="B116" t="s">
+        <v>54</v>
+      </c>
+      <c r="C116" t="s">
+        <v>79</v>
+      </c>
+      <c r="D116" t="s">
         <v>9</v>
       </c>
-      <c r="D113" t="s">
-        <v>15</v>
-      </c>
-      <c r="E113" t="s">
-        <v>46</v>
-      </c>
-      <c r="F113">
-        <v>3218.22</v>
-      </c>
-      <c r="G113" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
-        <v>278</v>
-      </c>
-      <c r="B114" t="s">
-        <v>82</v>
-      </c>
-      <c r="C114" t="s">
-        <v>97</v>
-      </c>
-      <c r="D114" t="s">
-        <v>24</v>
-      </c>
-      <c r="E114" t="s">
-        <v>42</v>
-      </c>
-      <c r="F114">
-        <v>303.69</v>
-      </c>
-      <c r="G114" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
-        <v>280</v>
-      </c>
-      <c r="B115" t="s">
-        <v>20</v>
-      </c>
-      <c r="C115" t="s">
-        <v>49</v>
-      </c>
-      <c r="D115" t="s">
-        <v>18</v>
-      </c>
-      <c r="E115" t="s">
-        <v>83</v>
-      </c>
-      <c r="F115" t="s">
-        <v>281</v>
-      </c>
-      <c r="G115" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
-        <v>283</v>
-      </c>
-      <c r="B116" t="s">
-        <v>82</v>
-      </c>
-      <c r="C116" t="s">
-        <v>121</v>
-      </c>
-      <c r="D116" t="s">
-        <v>10</v>
-      </c>
       <c r="E116" t="s">
-        <v>90</v>
-      </c>
-      <c r="F116" t="s">
-        <v>284</v>
+        <v>60</v>
+      </c>
+      <c r="F116" s="3" t="s">
+        <v>165</v>
       </c>
       <c r="G116" t="s">
-        <v>285</v>
+        <v>166</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
-        <v>286</v>
+      <c r="A117" s="1">
+        <v>44932</v>
       </c>
       <c r="B117" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C117" t="s">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="D117" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E117">
         <v>20</v>
       </c>
-      <c r="F117" t="s">
-        <v>287</v>
+      <c r="F117" s="3" t="s">
+        <v>167</v>
       </c>
       <c r="G117" t="s">
-        <v>288</v>
+        <v>168</v>
       </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>289</v>
+      <c r="A118" s="1">
+        <v>45073</v>
       </c>
       <c r="B118" t="s">
+        <v>7</v>
+      </c>
+      <c r="C118" t="s">
         <v>8</v>
       </c>
-      <c r="C118" t="s">
-        <v>9</v>
-      </c>
       <c r="D118" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E118" t="s">
-        <v>290</v>
-      </c>
-      <c r="F118" t="s">
-        <v>291</v>
+        <v>169</v>
+      </c>
+      <c r="F118" s="3" t="s">
+        <v>170</v>
       </c>
       <c r="G118">
         <v>71090.8</v>
       </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>63</v>
+      <c r="A119" s="1">
+        <v>45188</v>
       </c>
       <c r="B119" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C119" t="s">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="D119" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E119" t="s">
-        <v>42</v>
-      </c>
-      <c r="F119" t="s">
-        <v>292</v>
+        <v>29</v>
+      </c>
+      <c r="F119" s="3" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
-        <v>293</v>
+      <c r="A120" s="1">
+        <v>45080</v>
       </c>
       <c r="B120" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C120" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="D120" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E120" t="s">
-        <v>46</v>
-      </c>
-      <c r="F120">
+        <v>31</v>
+      </c>
+      <c r="F120" s="3">
         <v>2049.16</v>
       </c>
       <c r="G120" t="s">
-        <v>294</v>
+        <v>172</v>
       </c>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>295</v>
+      <c r="A121" s="1">
+        <v>45154</v>
       </c>
       <c r="B121" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C121" t="s">
-        <v>97</v>
+        <v>65</v>
       </c>
       <c r="D121" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E121" t="s">
-        <v>93</v>
-      </c>
-      <c r="F121">
+        <v>62</v>
+      </c>
+      <c r="F121" s="3">
         <v>4390.2700000000004</v>
       </c>
       <c r="G121" t="s">
-        <v>296</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G121" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Conclusão das Análises de KPIs
Conclusão das Análises de KPIs, como o faturamento total, a quantidade de vendas e o valor do ticket médio.
</commit_message>
<xml_diff>
--- a/data/dados_tratados.xlsx
+++ b/data/dados_tratados.xlsx
@@ -1,28 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\analise-vendas-excel\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{248DAA35-834A-496F-92BF-356043426EEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C2FF5F0-E2C0-4FA5-828E-410EC354968C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dados Tratados" sheetId="1" r:id="rId1"/>
-    <sheet name="Análises" sheetId="2" r:id="rId2"/>
-    <sheet name="Dashboard" sheetId="3" r:id="rId3"/>
+    <sheet name="Detalhes1" sheetId="4" state="hidden" r:id="rId2"/>
+    <sheet name="Análises" sheetId="2" r:id="rId3"/>
+    <sheet name="Dashboard" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dados Tratados'!$A$2:$G$123</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="12" r:id="rId4"/>
+    <pivotCache cacheId="12" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="48">
   <si>
     <t>Data</t>
   </si>
@@ -180,6 +181,15 @@
   <si>
     <t>Evolução do Faturamento Mensal</t>
   </si>
+  <si>
+    <t>1 . O faturamento mensal atingiu seu pico em agosto (R$380.675,46), indicando possíveis influências de campanhas comerciais ou aumento pontual na demanda.</t>
+  </si>
+  <si>
+    <t>2. Foram observadas quedas significativas em abril (R$ 90.114,66) e novembro (R$ 80.338,96), possivelmente relacionadas à fatores sazonais.</t>
+  </si>
+  <si>
+    <t>Detalhes do Soma de Receita - Meses (Data): Jun</t>
+  </si>
 </sst>
 </file>
 
@@ -260,7 +270,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="28">
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -441,11 +454,11 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US"/>
+              <a:rPr lang="en-US" b="1"/>
               <a:t>Evolução do Faturamento</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="en-US" baseline="0"/>
+              <a:rPr lang="en-US" b="1" baseline="0"/>
               <a:t> Mensal em 2023</a:t>
             </a:r>
           </a:p>
@@ -788,7 +801,9 @@
       <c:spPr>
         <a:noFill/>
         <a:ln>
-          <a:noFill/>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
         </a:ln>
         <a:effectLst/>
       </c:spPr>
@@ -1502,16 +1517,16 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>485775</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>4762</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>539</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>184479</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>359973</xdr:colOff>
       <xdr:row>25</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:rowOff>539</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3729,13 +3744,13 @@
     <dataField name="Soma de Receita" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="14">
-    <format dxfId="26">
+    <format dxfId="27">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="25">
+    <format dxfId="26">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="23">
+    <format dxfId="24">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="1">
@@ -3744,7 +3759,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="21">
+    <format dxfId="22">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="1">
@@ -3753,7 +3768,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
+    <format dxfId="20">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="1">
@@ -3762,7 +3777,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
+    <format dxfId="18">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="1">
@@ -3771,7 +3786,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="15">
+    <format dxfId="16">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="1">
@@ -3780,7 +3795,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="13">
+    <format dxfId="14">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="1">
@@ -3789,7 +3804,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="11">
+    <format dxfId="12">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="1">
@@ -3798,7 +3813,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="9">
+    <format dxfId="10">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="1">
@@ -3807,7 +3822,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="8">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="1">
@@ -3816,7 +3831,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="5">
+    <format dxfId="6">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="1">
@@ -3825,7 +3840,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="3">
+    <format dxfId="4">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="1">
@@ -3834,7 +3849,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="2">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="1">
@@ -3865,6 +3880,22 @@
     </ext>
   </extLst>
 </pivotTableDefinition>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B48DC75E-31D2-4CE8-8832-F3B6414A414D}" name="Tabela1" displayName="Tabela1" ref="A3:G14" totalsRowShown="0">
+  <autoFilter ref="A3:G14" xr:uid="{B48DC75E-31D2-4CE8-8832-F3B6414A414D}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{8F263DA3-B4AA-4FC5-8D25-5E8A900EC0AA}" name="Data" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{A54017AF-4388-4875-B62D-5100BEAF89A6}" name="Produto"/>
+    <tableColumn id="3" xr3:uid="{A73FF01D-D171-4AB8-B5B6-6C7DBE5D854F}" name="Região"/>
+    <tableColumn id="4" xr3:uid="{41F6B357-11B5-4542-BDA6-26F1631E5636}" name="Vendedor"/>
+    <tableColumn id="5" xr3:uid="{B46023A8-1EDD-465D-A154-6B882610EA59}" name="Quantidade"/>
+    <tableColumn id="6" xr3:uid="{C0E3DBF6-19EE-447E-95AB-7761F6843B93}" name="Preço Unitário"/>
+    <tableColumn id="7" xr3:uid="{746F4173-60BF-4272-A071-867538FA3E6F}" name="Receita"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7085,17 +7116,330 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C90171A-A64B-4A47-9F0F-E9F4B66FA6AC}">
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>45080</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4">
+        <v>6</v>
+      </c>
+      <c r="F4">
+        <v>2049.16</v>
+      </c>
+      <c r="G4">
+        <v>12294.96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>45081</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>1168.19</v>
+      </c>
+      <c r="G5">
+        <v>2336.38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>45082</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6">
+        <v>10</v>
+      </c>
+      <c r="F6">
+        <v>3923.26</v>
+      </c>
+      <c r="G6">
+        <v>39232.600000000006</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>45086</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7">
+        <v>4513.8999999999996</v>
+      </c>
+      <c r="G7">
+        <v>13541.699999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>45091</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8">
+        <v>10</v>
+      </c>
+      <c r="F8">
+        <v>2016.18</v>
+      </c>
+      <c r="G8">
+        <v>20161.8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>45091</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9">
+        <v>10</v>
+      </c>
+      <c r="F9">
+        <v>807.99</v>
+      </c>
+      <c r="G9">
+        <v>8079.9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>45091</v>
+      </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10">
+        <v>14</v>
+      </c>
+      <c r="F10">
+        <v>1401.69</v>
+      </c>
+      <c r="G10">
+        <v>19623.66</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>45093</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11">
+        <v>20</v>
+      </c>
+      <c r="F11">
+        <v>2505.5500000000002</v>
+      </c>
+      <c r="G11">
+        <v>50111</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>45097</v>
+      </c>
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12">
+        <v>3</v>
+      </c>
+      <c r="F12">
+        <v>573.21</v>
+      </c>
+      <c r="G12">
+        <v>1719.63</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>45101</v>
+      </c>
+      <c r="B13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13">
+        <v>8</v>
+      </c>
+      <c r="F13">
+        <v>4961.6000000000004</v>
+      </c>
+      <c r="G13">
+        <v>39692.800000000003</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>45106</v>
+      </c>
+      <c r="B14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14">
+        <v>18</v>
+      </c>
+      <c r="F14">
+        <v>1424.69</v>
+      </c>
+      <c r="G14">
+        <v>25644.420000000002</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56EE8C4F-4510-4B71-BD29-9F0FBEB655ED}">
-  <dimension ref="B5:E21"/>
+  <dimension ref="B4:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.5703125" customWidth="1"/>
+    <col min="7" max="7" width="31.140625" customWidth="1"/>
+    <col min="14" max="14" width="12.28515625" customWidth="1"/>
+    <col min="15" max="15" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="G4" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
         <v>40</v>
       </c>
@@ -7105,11 +7449,11 @@
       <c r="D5" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="6">
         <f>SUM('Dados Tratados'!G3:G122)</f>
         <v>2341703.4100000015</v>
@@ -7122,8 +7466,11 @@
         <f>B6/C6</f>
         <v>1984.4944152542387</v>
       </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="10" t="s">
         <v>43</v>
       </c>
@@ -7131,7 +7478,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="9" t="s">
         <v>28</v>
       </c>
@@ -7139,7 +7486,7 @@
         <v>199573.19000000003</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" s="9" t="s">
         <v>29</v>
       </c>
@@ -7147,7 +7494,7 @@
         <v>169251.27</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B11" s="9" t="s">
         <v>30</v>
       </c>
@@ -7155,7 +7502,7 @@
         <v>163357.34999999998</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="9" t="s">
         <v>31</v>
       </c>
@@ -7163,7 +7510,7 @@
         <v>90114.66</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" s="9" t="s">
         <v>32</v>
       </c>
@@ -7171,7 +7518,7 @@
         <v>160544.88999999998</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
         <v>33</v>
       </c>
@@ -7179,7 +7526,7 @@
         <v>232438.85</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="9" t="s">
         <v>34</v>
       </c>
@@ -7187,7 +7534,7 @@
         <v>207404.83999999997</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="9" t="s">
         <v>35</v>
       </c>
@@ -7241,7 +7588,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAD78F76-FE33-44D5-B879-616F6349FAC8}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>